<commit_message>
feat: Add PACIPA-MGP F01 complaint submission form and corresponding tests
- Created XML form for PACIPA-MGP F01 - Dépôt de plainte with multilingual support (French, Haoussa, Zarma).
- Implemented OdkF01MappingTest to validate complaint submission mapping.
- Added logic to handle site identification and complaints without associated sites.
</commit_message>
<xml_diff>
--- a/mgp-mobile/forms/xlsform/pacipa_mgp_f01_depot_plainte_v1.xlsx
+++ b/mgp-mobile/forms/xlsform/pacipa_mgp_f01_depot_plainte_v1.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="survey" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="choices" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M56"/>
+  <dimension ref="A1:M51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -590,7 +590,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SECTION 1 — Identification</t>
+          <t>SECTION 1 - Identification</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -606,6 +606,7 @@
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -640,37 +641,42 @@
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>select_one region</t>
+          <t>select_one oui_non</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>region</t>
+          <t>plainte_hors_site</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Région</t>
+          <t>Plainte hors-site (sans site associé) ?</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Yankin</t>
+          <t>Kara baya da wurin aikin ?</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Zaɲey</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+          <t>Lahari ka mana do zarma?</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Cocher si la plainte n'est liée à aucun site PACIPA.</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -683,30 +689,34 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>select_one departement</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>departement</t>
+          <t>site_id</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Département</t>
+          <t>Identifiant du site PACIPA</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Gundumar</t>
+          <t>Lambar wurin PACIPA</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Faaba</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
+          <t>Site ID PACIPA</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Saisir l'ID du site PACIPA. La localisation est déduite automatiquement côté serveur.</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
           <t>yes</t>
@@ -717,41 +727,46 @@
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>${region} != ''</t>
+          <t>${plainte_hors_site} != 'oui'</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>select_one commune</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>commune</t>
+          <t>site_libre</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Commune</t>
+          <t>Préciser le lieu (si hors-site)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Birni</t>
+          <t>Faɗi wurin</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Koome</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
+          <t>Faaba zarma</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Ex: Marché de Dosso</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -759,295 +774,298 @@
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>${departement} != ''</t>
+          <t>${plainte_hors_site} = 'oui'</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>select_one localite</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>localite</t>
+          <t>id_plainte</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Localité / Village</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Gari</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Katoo</t>
-        </is>
-      </c>
+          <t>Numéro de plainte</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>${commune} != ''</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>concat(if(${plainte_hors_site} = 'oui','HS',${site_id}),'-',format-date(today(),'%Y'),'-',substr(uuid(),0,8))</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>select_one site</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>site</t>
+          <t>note_id</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Site PACIPA</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Wurin aikin PACIPA</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>PACIPA zarma</t>
-        </is>
-      </c>
+          <t>Numéro attribué :</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>minimal</t>
-        </is>
-      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>${localite} != '' and ${plainte_hors_site} = 'non'</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>${id_plainte}</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>select_one oui_non</t>
+          <t>end_group</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>plainte_hors_site</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Plainte hors-site (sans site associé) ?</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Kara baya da wurin aikin ?</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Lahari ka mana do zarma?</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>La plainte n'est pas liée à un site PACIPA spécifique</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+          <t>grp_identification</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>site_libre</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Préciser le site (si non listé)</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Faɗi wurin (idan ba a lissafa ba)</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Faaba zarma (idan a mana tara)</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Ex: "Marché de Dosso"</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>${plainte_hors_site} = 'oui'</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>id_plainte</t>
+          <t>grp_plaignant</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Numéro de plainte</t>
+          <t>SECTION 2 - Identité du plaignant</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>concat(regex(${region},'.*'), '-', regex(${departement},'.*'), '-', regex(${commune},'.*'), '-', format-date(today(),'%Y'), '-', uuid())</t>
-        </is>
-      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>${type} != 'type8'</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>select_one oui_non</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>note_id</t>
+          <t>anonymat</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Numéro attribué :</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
+          <t>Le plaignant souhaite rester anonyme ?</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Masu iɗa sai dai a ɓoye su ?</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Boro go hãy koy alhaali zarma?</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Consentement explicite requis avant toute identification.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>${id_plainte}</t>
-        </is>
-      </c>
+      <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>end_group</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>grp_identification</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
+          <t>nom_prenom</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Nom et Prénom</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Suna da sunan mahaifi</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Turo ga ceeci</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>${anonymat} = 'non'</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>age</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Âge (années)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Shekaru</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Jiiri (ceeci)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Âge du plaignant en années</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>number &gt; 0 and number &lt; 120</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>select_one genre</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>grp_plaignant</t>
+          <t>genre</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SECTION 2 — Identité du plaignant</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+          <t>Genre</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Jinsi</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Jinsi</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
@@ -1057,34 +1075,30 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>select_one oui_non</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>anonymat</t>
+          <t>lieu_residence</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Le plaignant souhaite rester anonyme ?</t>
+          <t>Lieu de résidence</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Masu iɗa sai dai a ɓoye su ?</t>
+          <t>Wurin zama</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Boro go hãy koy alhaali zarma?</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Consentement explicite requis avant toute identification.</t>
-        </is>
-      </c>
+          <t>Zama wane</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>yes</t>
@@ -1095,6 +1109,7 @@
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1104,290 +1119,295 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>nom_prenom</t>
+          <t>contact</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Nom et Prénom</t>
+          <t>Contact téléphone (+227XXXXXXXX)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Suna da sunan mahaifi</t>
+          <t>Lambar waya (+227XXXXXXXX)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Turo ga ceeci</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
+          <t>Tele zarma (+227XXXXXXXX)</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Format Niger +227 suivi de 8 chiffres</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>${anonymat} = 'non'</t>
-        </is>
-      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>regex(., '^\+227[0-9]{8}$')</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Format : +227XXXXXXXX</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>end_group</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>age</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Âge (années)</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Shekaru</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Jiiri (ceeci)</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Âge du plaignant en années</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>grp_plaignant</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>number &gt; 0 and number &lt; 120</t>
-        </is>
-      </c>
+      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>select_one genre</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>genre</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Genre</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Jinsi</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Jinsi</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-    </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>lieu_residence</t>
+          <t>grp_plainte</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Lieu de résidence</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Wurin zama</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Zama wane</t>
-        </is>
-      </c>
+          <t>SECTION 3 - Objet de la plainte</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one type_plainte</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>type</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Contact téléphone (+227XXXXXXXX)</t>
+          <t>Type de plainte</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Lambar waya (+227XXXXXXXX)</t>
+          <t>Nau'in kara</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Tele zarma (+227XXXXXXXX)</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Format Niger +227 suivi de 8 chiffres</t>
-        </is>
-      </c>
+          <t>Lahari zarma</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>regex(., '^\+227[0-9]{8}$')</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>Format : +227XXXXXXXX</t>
-        </is>
-      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>end_group</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>grp_plaignant</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
+          <t>note_vbg</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>⚠️ TYPE 8 - VBG/EAS/HS : Rendez-vous sur le formulaire F03 dédié. NE PAS continuer ce formulaire.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>⚠️ Nau'i 8 - VBG : Zuwa F03.</t>
+        </is>
+      </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>${type} = 'type8'</t>
+        </is>
+      </c>
       <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>personne_visee</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Personne ou structure visée par la plainte</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Wanda ake kara a kansa</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Boro lahari zarma</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>${type} != 'type8'</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>grp_plainte</t>
+          <t>description</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>SECTION 3 — Objet de la plainte</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
+          <t>Description détaillée de la plainte</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Bayani game da kara</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Lahari zarma bayani</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Décrivez les faits de manière précise et chronologique</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>field-list</t>
+          <t>multiline</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>${type} != 'type8'</t>
+        </is>
+      </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>select_one type_plainte</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>type</t>
+          <t>date_faits</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Type de plainte</t>
+          <t>Date des faits</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Nau'in kara</t>
+          <t>Ranar abin da ya faru</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Lahari zarma</t>
+          <t>Zarma (araw lahari)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -1399,31 +1419,40 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>${type} != 'type8'</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin_repeat</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>note_vbg</t>
+          <t>temoins</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>⚠️ TYPE 8 — VBG/EAS/HS : Vous serez redirigé vers le formulaire F03 dédié. NE PAS continuer ce formulaire.</t>
+          <t>Témoins (optionnel)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>⚠️ Nau'i 8 — VBG : Zuwa F03.</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr"/>
+          <t>Shaidu</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Zarma (temoins)</t>
+        </is>
+      </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
@@ -1431,10 +1460,11 @@
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
-          <t>${type} = 'type8'</t>
+          <t>${type} != 'type8'</t>
         </is>
       </c>
       <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1444,28 +1474,28 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>personne_visee</t>
+          <t>temoin_nom</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Personne ou structure visée par la plainte</t>
+          <t>Nom du témoin</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Wanda ake kara a kansa</t>
+          <t>Suna shaidu</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Boro lahari zarma</t>
+          <t>Zarma temoin suna</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
@@ -1473,6 +1503,7 @@
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1482,207 +1513,160 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>temoin_contact</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Description détaillée de la plainte</t>
+          <t>Contact du témoin</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Bayani game da kara</t>
+          <t>Lambar waya shaidu</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Lahari zarma bayani</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Décrivez les faits de manière précise et chronologique</t>
-        </is>
-      </c>
+          <t>Zarma temoin tele</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>end_repeat</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>date_faits</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Date des faits</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Ranar abin da ya faru</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Zarma (araw lahari)</t>
-        </is>
-      </c>
+          <t>temoins</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>begin_repeat</t>
+          <t>end_group</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>temoins</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Témoins (optionnel)</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Shaidu</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Zarma (temoins)</t>
-        </is>
-      </c>
+          <t>grp_plainte</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>temoin_nom</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Nom du témoin</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Suna shaidu</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Zarma temoin suna</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>temoin_contact</t>
+          <t>grp_canal</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Contact du témoin</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Lambar waya shaidu</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Zarma temoin tele</t>
-        </is>
-      </c>
+          <t>SECTION 4 - Canal de réception</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>${type} != 'type8'</t>
+        </is>
+      </c>
       <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>end_repeat</t>
+          <t>select_one canal</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>temoins</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
+          <t>canal</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Canal de réception de la plainte</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Hanyar karɓar kara</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Lahari zarma ganda</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Comment la plainte a-t-elle été reçue ?</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1692,7 +1676,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>grp_plainte</t>
+          <t>grp_canal</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -1705,6 +1689,7 @@
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1714,12 +1699,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>grp_canal</t>
+          <t>grp_pj</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SECTION 4 — Canal de réception</t>
+          <t>SECTION 5 - Pièces jointes (optionnel)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1733,44 +1718,44 @@
       </c>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>${type} != 'type8'</t>
+        </is>
+      </c>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>select_one canal</t>
+          <t>image</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>canal</t>
+          <t>photo1</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Canal de réception de la plainte</t>
+          <t>Photo 1 (optionnel)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Hanyar karɓar kara</t>
+          <t>Hoto 1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Lahari zarma ganda</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Comment la plainte a-t-elle été reçue ?</t>
-        </is>
-      </c>
+          <t>Zarma photo 1</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H42" t="inlineStr"/>
@@ -1778,181 +1763,269 @@
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>end_group</t>
+          <t>image</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>grp_canal</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
+          <t>photo2</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Photo 2 (optionnel)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Hoto 2</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Zarma photo 2</t>
+        </is>
+      </c>
       <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>begin_group</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
+      <c r="M43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
         <is>
           <t>grp_pj</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>SECTION 5 — Pièces jointes (optionnel)</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>image</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>photo1</t>
+          <t>grp_confirmation</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Photo 1 (optionnel)</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Hoto 1</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Zarma photo 1</t>
-        </is>
-      </c>
+          <t>SECTION 6 - Confirmation et signature</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>${type} != 'type8'</t>
+        </is>
+      </c>
       <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>image</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>photo2</t>
+          <t>note_resume</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Photo 2 (optionnel)</t>
+          <t>Récapitulatif — Type : ${type} · Plaignant : ${nom_prenom} (${age} ans) · Faits du ${date_faits} · Site : ${site_id}. Vérifiez avant de soumettre.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Hoto 2</t>
+          <t>Duba bayanan da ka shigar kafin tura.</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Zarma photo 2</t>
+          <t>Gaa koy alhaali zarma.</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>end_group</t>
+          <t>geopoint</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>grp_pj</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
+          <t>gps</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Position GPS (automatique)</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Matsayin GPS</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>GPS zarma</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Position au moment de l'enregistrement</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>placement-map</t>
+        </is>
+      </c>
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>datetime</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>timestamp_enreg</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Date et heure d'enregistrement</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Ranar da lokacin yin rubutu</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Zarma araw</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Automatique</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>now()</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>image</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>grp_confirmation</t>
+          <t>signature_agent</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>SECTION 6 — Confirmation et signature</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
+          <t>Signature du chargé d'enregistrement</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Sa'in Jami'in</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Zarma agent sa'a</t>
+        </is>
+      </c>
       <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>field-list</t>
+          <t>signature</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
@@ -1964,29 +2037,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>end_group</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>note_resume</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Vérifiez les informations saisies avant de soumettre.</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Duba bayanan da ka shigar kafin tura.</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Gaa koy alhaali zarma.</t>
-        </is>
-      </c>
+          <t>grp_confirmation</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
@@ -1995,184 +2056,6 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>geopoint</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>gps</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Position GPS (automatique)</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Matsayin GPS</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>GPS zarma</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>Position au moment de l'enregistrement</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>placement-map</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>datetime</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>timestamp_enreg</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Date et heure d'enregistrement</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Ranar da lokacin yin rubutu</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Zarma araw</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>Automatique</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>calculate</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>calculate</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>ts_calc</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>now()</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>draw</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>signature_agent</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Signature du chargé d'enregistrement</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>Sa'in Jami'in</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Zarma agent sa'a</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>grp_confirmation</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2185,7 +2068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2272,486 +2155,486 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>region</t>
+          <t>genre</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>agadez</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Agadez</t>
+          <t>Féminin</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Agadez</t>
+          <t>Mata</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Agadez</t>
+          <t>Haw</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>region</t>
+          <t>genre</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>diffa</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Diffa</t>
+          <t>Masculin</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Diffa</t>
+          <t>Maza</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Diffa</t>
+          <t>Wane</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>region</t>
+          <t>type_plainte</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>dosso</t>
+          <t>type1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Dosso</t>
+          <t>Type 1 - Inaccessibilité aux informations</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Dosso</t>
+          <t>Nau'i 1 - Babu bayani</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Dosso</t>
+          <t>Zarma nau'i 1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>region</t>
+          <t>type_plainte</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>maradi</t>
+          <t>type2</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Maradi</t>
+          <t>Type 2 - Exécution des marchés</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Maradi</t>
+          <t>Nau'i 2 - Aiki da kwangilar</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Maradi</t>
+          <t>Zarma nau'i 2</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>region</t>
+          <t>type_plainte</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>niamey</t>
+          <t>type3</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Niamey</t>
+          <t>Type 3 - Travaux de réhabilitation</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Niamey</t>
+          <t>Nau'i 3 - Aikin gina</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Niamey</t>
+          <t>Zarma nau'i 3</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>region</t>
+          <t>type_plainte</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>tahoua</t>
+          <t>type4</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tahoua</t>
+          <t>Type 4 - Conditions de travail</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Tahoua</t>
+          <t>Nau'i 4 - Yanayin aiki</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Tahoua</t>
+          <t>Zarma nau'i 4</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>region</t>
+          <t>type_plainte</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>tillaberi</t>
+          <t>type5</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Tillabéri</t>
+          <t>Type 5 - Pertes/affectation de biens</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Tillabéri</t>
+          <t>Nau'i 5 - Asara/raba dukiya</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Tillabéri</t>
+          <t>Zarma nau'i 5</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>region</t>
+          <t>type_plainte</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>zinder</t>
+          <t>type6</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Zinder</t>
+          <t>Type 6 - Octroi d'équipements</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Zinder</t>
+          <t>Nau'i 6 - Ba da kayan aiki</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Zinder</t>
+          <t>Zarma nau'i 6</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>genre</t>
+          <t>type_plainte</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>type7</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Féminin</t>
+          <t>Type 7 - Formations</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Mata</t>
+          <t>Nau'i 7 - Horo</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Haw</t>
+          <t>Zarma nau'i 7</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>genre</t>
+          <t>type_plainte</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>type8</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Masculin</t>
+          <t>Type 8 - VBG / EAS / HS / VCE ⚠️</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Maza</t>
+          <t>Nau'i 8 - VBG / EAS / HS</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Wane</t>
+          <t>Zarma nau'i 8</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>type_plainte</t>
+          <t>canal</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>type1</t>
+          <t>en_personne</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Type 1 — Inaccessibilité aux informations</t>
+          <t>En personne</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Nau'i 1 — Babu bayani</t>
+          <t>Kai tsaye</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Zarma nau'i 1</t>
+          <t>Zarma en personne</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>type_plainte</t>
+          <t>canal</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>type2</t>
+          <t>telephone</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Type 2 — Exécution des marchés</t>
+          <t>Téléphone</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Nau'i 2 — Aiki da kwangilar</t>
+          <t>Waya</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Zarma nau'i 2</t>
+          <t>Zarma telephone</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>type_plainte</t>
+          <t>canal</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>type3</t>
+          <t>sms</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Type 3 — Travaux de réhabilitation</t>
+          <t>SMS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Nau'i 3 — Aikin gina</t>
+          <t>SMS</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Zarma nau'i 3</t>
+          <t>SMS</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>type_plainte</t>
+          <t>canal</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>type4</t>
+          <t>whatsapp</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Type 4 — Conditions de travail</t>
+          <t>WhatsApp</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Nau'i 4 — Yanayin aiki</t>
+          <t>WhatsApp</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Zarma nau'i 4</t>
+          <t>WhatsApp</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>type_plainte</t>
+          <t>canal</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>type5</t>
+          <t>courrier</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Type 5 — Pertes/affectation de biens</t>
+          <t>Courrier postal</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Nau'i 5 — Asara/raba dukiya</t>
+          <t>Wasiƙa</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Zarma nau'i 5</t>
+          <t>Zarma courrier</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>type_plainte</t>
+          <t>canal</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>type6</t>
+          <t>email</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Type 6 — Octroi d'équipements</t>
+          <t>Email / Courriel</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Nau'i 6 — Ba da kayan aiki</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Zarma nau'i 6</t>
+          <t>Email</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>type_plainte</t>
+          <t>canal</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>type7</t>
+          <t>boite_reclamation</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Type 7 — Formations</t>
+          <t>Boîte à réclamations</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Nau'i 7 — Horo</t>
+          <t>Akwatin kara</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Zarma nau'i 7</t>
+          <t>Zarma boite</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>type_plainte</t>
+          <t>canal</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>type8</t>
+          <t>ligne_verte</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Type 8 — VBG / EAS / HS / VCE ⚠️</t>
+          <t>Ligne verte (numéro vert)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Nau'i 8 — VBG / EAS / HS</t>
+          <t>Layin kore</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Zarma nau'i 8</t>
+          <t>Zarma ligne verte</t>
         </is>
       </c>
     </row>
@@ -2763,236 +2646,20 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>en_personne</t>
+          <t>auto_saisine</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>En personne</t>
+          <t>Auto-saisine (presse/rapport)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Kai tsaye</t>
+          <t>Auto-saisine</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
-        <is>
-          <t>Zarma en personne</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>canal</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>telephone</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Téléphone</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Waya</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Zarma telephone</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>canal</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>sms</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>SMS</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>canal</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>whatsapp</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>WhatsApp</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>WhatsApp</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>WhatsApp</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>canal</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>courrier</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Courrier postal</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Wasiƙa</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Zarma courrier</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>canal</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>email</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Email / Courriel</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>canal</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>boite_reclamation</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Boîte à réclamations</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Akwatin kara</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Zarma boite</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>canal</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>ligne_verte</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Ligne verte (numéro vert)</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Layin kore</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Zarma ligne verte</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>canal</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>auto_saisine</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Auto-saisine (presse/rapport)</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Auto-saisine</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
         <is>
           <t>Zarma auto-saisine</t>
         </is>
@@ -3052,7 +2719,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PACIPA-MGP F01 — Dépôt de plainte</t>
+          <t>PACIPA-MGP F01 - Dépôt de plainte</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>